<commit_message>
[Update] GamePLay팝업 상세 구현
[수정]
- StageStart, StageFailed, StageClear 디자인 변경 및 내용 추가
 StageStart: 목표 골드 시각화
 StageFailed: 플레이 타임만 표시
 StageClear: 클리어 타임, 총 점수 표기 및 상세 점수내역 토글기능 추가
- StageClear 조건 설정에 따라 버튼 클릭시 Context.Gold 차감 후 Clear팝업 출력
- Planet 스폰 주기 수정 및 시간 표기용 MathUtility 메서드 추가
</commit_message>
<xml_diff>
--- a/JsonConverter/ExcelFiles/Stage.xlsx
+++ b/JsonConverter/ExcelFiles/Stage.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="16524" windowHeight="8400"/>
+    <workbookView windowWidth="23040" windowHeight="9000"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -92,7 +92,7 @@
     <t>Stage_normal_00</t>
   </si>
   <si>
-    <t>Training Zone</t>
+    <t>모의 시뮬레이션</t>
   </si>
   <si>
     <t>true</t>
@@ -104,7 +104,7 @@
     <t>Stage_normal_01</t>
   </si>
   <si>
-    <t>First Frontier</t>
+    <t>첫 임무</t>
   </si>
   <si>
     <t>false</t>
@@ -116,7 +116,7 @@
     <t>Stage_normal_02</t>
   </si>
   <si>
-    <t>Asteroid Belt</t>
+    <t>소행성대</t>
   </si>
   <si>
     <t>Planet_small_01,Planet_small_02,Planet_small_03,Planet_small_04,Planet_small_05,Planet_small_06</t>
@@ -125,7 +125,7 @@
     <t>Stage_normal_03</t>
   </si>
   <si>
-    <t>Deep Void</t>
+    <t>외곽 지대</t>
   </si>
   <si>
     <t>Planet_small_02,Planet_small_03,Planet_small_04,Planet_small_05,Planet_small_06</t>
@@ -134,7 +134,7 @@
     <t>Stage_normal_04</t>
   </si>
   <si>
-    <t>Super Cluster</t>
+    <t>성운 항로</t>
   </si>
   <si>
     <t>Planet_small_02,Planet_small_03,Planet_small_04,Planet_small_05,Planet_small_06,Planet_small_07</t>
@@ -143,7 +143,7 @@
     <t>Stage_normal_05</t>
   </si>
   <si>
-    <t>Nebula Trade Route</t>
+    <t>심우주</t>
   </si>
   <si>
     <t>Planet_small_03,Planet_small_04,Planet_small_05,Planet_small_07,Planet_medium_01,Planet_medium_02</t>
@@ -152,7 +152,7 @@
     <t>Stage_normal_06</t>
   </si>
   <si>
-    <t>The Outer Rim</t>
+    <t>우주 교차로</t>
   </si>
   <si>
     <t>Planet_small_03,Planet_small_04,Planet_small_06,Planet_small_07,Planet_medium_01,Planet_medium_02,Planet_medium_03</t>
@@ -161,7 +161,7 @@
     <t>Stage_normal_07</t>
   </si>
   <si>
-    <t>Cosmic Intersection</t>
+    <t>청색 성단</t>
   </si>
   <si>
     <t>Planet_small_03,Planet_small_05,Planet_small_07,Planet_medium_01,Planet_medium_02,Planet_medium_03,Planet_medium_04</t>
@@ -170,7 +170,7 @@
     <t>Stage_normal_08</t>
   </si>
   <si>
-    <t>Galactic Frontier</t>
+    <t>은하 개척지</t>
   </si>
   <si>
     <t>Planet_small_02,Planet_small_04,Planet_medium_01,Planet_medium_02,Planet_medium_04,Planet_medium_05</t>
@@ -179,7 +179,7 @@
     <t>Stage_normal_09</t>
   </si>
   <si>
-    <t>Supercluster Core</t>
+    <t>초성단 핵심부</t>
   </si>
   <si>
     <t>Planet_small_01,Planet_small_03,Planet_small_05,Planet_small_07,Planet_medium_01,Planet_medium_03,Planet_medium_05,Planet_Large_01</t>
@@ -188,7 +188,7 @@
     <t>Stage_normal_10</t>
   </si>
   <si>
-    <t>The Infinite Void</t>
+    <t>공허 심부</t>
   </si>
   <si>
     <t>Planet_small_02,Planet_small_05,Planet_small_07,Planet_medium_03,Planet_medium_04,Planet_medium_05,Planet_Large_01,Planet_Large_02</t>
@@ -807,14 +807,11 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
@@ -1445,7 +1442,7 @@
         <v>3</v>
       </c>
       <c r="D4">
-        <v>36</v>
+        <v>48</v>
       </c>
       <c r="E4">
         <v>0.05</v>
@@ -1468,10 +1465,10 @@
         <v>25</v>
       </c>
       <c r="C5">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D5">
-        <v>36</v>
+        <v>48</v>
       </c>
       <c r="E5">
         <v>0.05</v>
@@ -1494,10 +1491,10 @@
         <v>29</v>
       </c>
       <c r="C6">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D6">
-        <v>36</v>
+        <v>48</v>
       </c>
       <c r="E6">
         <v>0.075</v>
@@ -1516,14 +1513,14 @@
       <c r="A7" t="s">
         <v>31</v>
       </c>
-      <c r="B7" s="2" t="s">
+      <c r="B7" t="s">
         <v>32</v>
       </c>
       <c r="C7">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D7">
-        <v>32</v>
+        <v>44</v>
       </c>
       <c r="E7">
         <v>0.075</v>
@@ -1542,14 +1539,14 @@
       <c r="A8" t="s">
         <v>34</v>
       </c>
-      <c r="B8" s="2" t="s">
+      <c r="B8" t="s">
         <v>35</v>
       </c>
       <c r="C8">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D8">
-        <v>32</v>
+        <v>44</v>
       </c>
       <c r="E8">
         <v>0.1</v>
@@ -1568,14 +1565,14 @@
       <c r="A9" t="s">
         <v>37</v>
       </c>
-      <c r="B9" s="2" t="s">
+      <c r="B9" t="s">
         <v>38</v>
       </c>
       <c r="C9">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D9">
-        <v>30</v>
+        <v>42</v>
       </c>
       <c r="E9">
         <v>0.1</v>
@@ -1594,14 +1591,14 @@
       <c r="A10" t="s">
         <v>40</v>
       </c>
-      <c r="B10" s="2" t="s">
+      <c r="B10" t="s">
         <v>41</v>
       </c>
       <c r="C10">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D10">
-        <v>28</v>
+        <v>40</v>
       </c>
       <c r="E10">
         <v>0.125</v>
@@ -1620,14 +1617,14 @@
       <c r="A11" t="s">
         <v>43</v>
       </c>
-      <c r="B11" s="2" t="s">
+      <c r="B11" t="s">
         <v>44</v>
       </c>
       <c r="C11">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="D11">
-        <v>28</v>
+        <v>38</v>
       </c>
       <c r="E11">
         <v>0.175</v>
@@ -1646,14 +1643,14 @@
       <c r="A12" t="s">
         <v>46</v>
       </c>
-      <c r="B12" s="2" t="s">
+      <c r="B12" t="s">
         <v>47</v>
       </c>
       <c r="C12">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="D12">
-        <v>26</v>
+        <v>36</v>
       </c>
       <c r="E12">
         <v>0.235</v>
@@ -1672,14 +1669,14 @@
       <c r="A13" t="s">
         <v>49</v>
       </c>
-      <c r="B13" s="2" t="s">
+      <c r="B13" t="s">
         <v>50</v>
       </c>
       <c r="C13">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="D13">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="E13">
         <v>0.285</v>
@@ -1698,14 +1695,14 @@
       <c r="A14" t="s">
         <v>52</v>
       </c>
-      <c r="B14" s="2" t="s">
+      <c r="B14" t="s">
         <v>53</v>
       </c>
       <c r="C14">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D14">
-        <v>24</v>
+        <v>32</v>
       </c>
       <c r="E14">
         <v>0.35</v>

</xml_diff>